<commit_message>
feat: add player profile images and update player selection count UI
</commit_message>
<xml_diff>
--- a/static/images/jogadores/Informações de Jogador - Vale no Volei (respostas).xlsx
+++ b/static/images/jogadores/Informações de Jogador - Vale no Volei (respostas).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="57">
   <si>
     <t>Carimbo de data/hora</t>
   </si>
@@ -153,6 +153,33 @@
   </si>
   <si>
     <t>marcio-sa-jpeg</t>
+  </si>
+  <si>
+    <t>Lacerda</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1V3kaFaxYDDVvvbvTOZy-luJ26jP6LnaI</t>
+  </si>
+  <si>
+    <t>lacerda.jpeg</t>
+  </si>
+  <si>
+    <t>Carlos</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=14Pweb8TweWQ-bNUuL8dFFJqST2Me2cup</t>
+  </si>
+  <si>
+    <t>carlos.jpeg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giovana </t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1hNWOOUYsWMpEU4jjIdS-e46mNCbnF9Ky</t>
+  </si>
+  <si>
+    <t>giovana.jpeg</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
@@ -321,7 +348,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E13" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E16" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="5">
     <tableColumn name="Carimbo de data/hora" id="1"/>
     <tableColumn name="Qual seu nome de Jogador no Vale?" id="2"/>
@@ -759,18 +786,60 @@
       <c r="D13" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="7" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="14">
-      <c r="E14" s="11"/>
-    </row>
-    <row r="15">
-      <c r="E15" s="11"/>
-    </row>
-    <row r="16">
-      <c r="E16" s="11"/>
+    <row r="14" ht="22.5" customHeight="1">
+      <c r="A14" s="8">
+        <v>46148.56343212963</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="15" ht="22.5" customHeight="1">
+      <c r="A15" s="8">
+        <v>46148.59246189815</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16" ht="22.5" customHeight="1">
+      <c r="A16" s="8">
+        <v>46148.599649525466</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="17">
       <c r="E17" s="11"/>
@@ -803,9 +872,7 @@
       <c r="E26" s="11"/>
     </row>
     <row r="27">
-      <c r="E27" s="12" t="s">
-        <v>47</v>
-      </c>
+      <c r="E27" s="11"/>
     </row>
     <row r="28">
       <c r="E28" s="11"/>
@@ -814,7 +881,9 @@
       <c r="E29" s="11"/>
     </row>
     <row r="30">
-      <c r="E30" s="11"/>
+      <c r="E30" s="12" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="31">
       <c r="E31" s="11"/>
@@ -1064,6 +1133,15 @@
     </row>
     <row r="113">
       <c r="E113" s="11"/>
+    </row>
+    <row r="114">
+      <c r="E114" s="11"/>
+    </row>
+    <row r="115">
+      <c r="E115" s="11"/>
+    </row>
+    <row r="116">
+      <c r="E116" s="11"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1079,10 +1157,13 @@
     <hyperlink r:id="rId10" ref="D11"/>
     <hyperlink r:id="rId11" ref="D12"/>
     <hyperlink r:id="rId12" ref="D13"/>
+    <hyperlink r:id="rId13" ref="D14"/>
+    <hyperlink r:id="rId14" ref="D15"/>
+    <hyperlink r:id="rId15" ref="D16"/>
   </hyperlinks>
-  <drawing r:id="rId13"/>
+  <drawing r:id="rId16"/>
   <tableParts count="1">
-    <tablePart r:id="rId15"/>
+    <tablePart r:id="rId18"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: correct file extension for Marcio Sá's photo path in player data
</commit_message>
<xml_diff>
--- a/static/images/jogadores/Informações de Jogador - Vale no Volei (respostas).xlsx
+++ b/static/images/jogadores/Informações de Jogador - Vale no Volei (respostas).xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="60">
   <si>
     <t xml:space="preserve">Carimbo de data/hora</t>
   </si>
@@ -192,6 +192,12 @@
   </si>
   <si>
     <t xml:space="preserve">icaro.jpeg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">edu.jpeg</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
@@ -846,8 +852,19 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E18" s="7"/>
+    <row r="18" customFormat="false" ht="25.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="n">
+        <v>46148.6856365741</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E19" s="7"/>
@@ -884,7 +901,7 @@
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E30" s="7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
feat: add Andrew to player list and include corresponding profile image
</commit_message>
<xml_diff>
--- a/static/images/jogadores/Informações de Jogador - Vale no Volei (respostas).xlsx
+++ b/static/images/jogadores/Informações de Jogador - Vale no Volei (respostas).xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="64">
   <si>
     <t xml:space="preserve">Carimbo de data/hora</t>
   </si>
@@ -197,7 +197,19 @@
     <t xml:space="preserve">Edu</t>
   </si>
   <si>
+    <t xml:space="preserve">https://drive.google.com/open?id=1yMfFFRWJX8R-DSQ3TK077fymTw0UYyUI</t>
+  </si>
+  <si>
     <t xml:space="preserve">edu.jpeg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andrew</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://drive.google.com/open?id=1Gs8G0fZraYGpzH9BXnakS_xEHdlDf96O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">andrew.jpeg</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
@@ -862,17 +874,36 @@
       <c r="C18" s="5" t="s">
         <v>10</v>
       </c>
+      <c r="D18" s="6" t="s">
+        <v>58</v>
+      </c>
       <c r="E18" s="7" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E19" s="7"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="n">
+        <v>46148.7556712963</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D20" s="6"/>
       <c r="E20" s="7"/>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D21" s="6"/>
       <c r="E21" s="7"/>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -901,7 +932,7 @@
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E30" s="7" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1180,6 +1211,8 @@
     <hyperlink ref="D15" r:id="rId14" display="https://drive.google.com/open?id=14Pweb8TweWQ-bNUuL8dFFJqST2Me2cup"/>
     <hyperlink ref="D16" r:id="rId15" display="https://drive.google.com/open?id=1hNWOOUYsWMpEU4jjIdS-e46mNCbnF9Ky"/>
     <hyperlink ref="D17" r:id="rId16" display="https://drive.google.com/open?id=1hNWOOUYsWMpEU4jjIdS-e46mNCbnF9Ky"/>
+    <hyperlink ref="D18" r:id="rId17" display="https://drive.google.com/open?id=1yMfFFRWJX8R-DSQ3TK077fymTw0UYyUI"/>
+    <hyperlink ref="D19" r:id="rId18" display="https://drive.google.com/open?id=1Gs8G0fZraYGpzH9BXnakS_xEHdlDf96O"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1189,7 +1222,7 @@
     <oddFooter/>
   </headerFooter>
   <tableParts>
-    <tablePart r:id="rId17"/>
+    <tablePart r:id="rId19"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add Jairo Davi player profile and associated image to static assets
</commit_message>
<xml_diff>
--- a/static/images/jogadores/Informações de Jogador - Vale no Volei (respostas).xlsx
+++ b/static/images/jogadores/Informações de Jogador - Vale no Volei (respostas).xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="66">
   <si>
     <t xml:space="preserve">Carimbo de data/hora</t>
   </si>
@@ -210,6 +210,12 @@
   </si>
   <si>
     <t xml:space="preserve">andrew.jpeg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jairo Davi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">davi.jpeg</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
@@ -898,9 +904,22 @@
         <v>62</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D20" s="6"/>
-      <c r="E20" s="7"/>
+    <row r="20" customFormat="false" ht="24.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="n">
+        <v>46149.6553472222</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D21" s="6"/>
@@ -932,7 +951,7 @@
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E30" s="7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1213,6 +1232,7 @@
     <hyperlink ref="D17" r:id="rId16" display="https://drive.google.com/open?id=1hNWOOUYsWMpEU4jjIdS-e46mNCbnF9Ky"/>
     <hyperlink ref="D18" r:id="rId17" display="https://drive.google.com/open?id=1yMfFFRWJX8R-DSQ3TK077fymTw0UYyUI"/>
     <hyperlink ref="D19" r:id="rId18" display="https://drive.google.com/open?id=1Gs8G0fZraYGpzH9BXnakS_xEHdlDf96O"/>
+    <hyperlink ref="D20" r:id="rId19" display="https://drive.google.com/open?id=1Gs8G0fZraYGpzH9BXnakS_xEHdlDf96O"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1222,7 +1242,7 @@
     <oddFooter/>
   </headerFooter>
   <tableParts>
-    <tablePart r:id="rId19"/>
+    <tablePart r:id="rId20"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>